<commit_message>
progress: 34 village workbooks (randomwalk-TRX50-WS 2026-10-09T15:30:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Arikathurai_13.34632_80.126.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Arikathurai_13.34632_80.126.xlsx
@@ -446,11 +446,6 @@
           <t>10</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -458,11 +453,6 @@
           <t>11</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -470,11 +460,6 @@
           <t>12</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 3A, 3B, 4, 5A, 5B</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -482,11 +467,6 @@
           <t>13</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 2A, 2B, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -494,11 +474,6 @@
           <t>14</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -506,11 +481,6 @@
           <t>15</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -518,11 +488,6 @@
           <t>16</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -530,11 +495,6 @@
           <t>17</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -542,11 +502,6 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B, 2C, 2D, 2E, 3</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -554,11 +509,6 @@
           <t>19</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1, 1B2, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -566,11 +516,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -578,11 +523,6 @@
           <t>20</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C1, 10C2, 10C3, 11, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -590,11 +530,6 @@
           <t>21</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16A, 16B, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -602,11 +537,6 @@
           <t>22</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -614,11 +544,6 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -626,11 +551,6 @@
           <t>24</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -638,11 +558,6 @@
           <t>25</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>1, 10, 2, 3, 4, 5A, 5B, 6, 7, 8A, 8B, 8C, 9</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -650,11 +565,6 @@
           <t>26</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -662,11 +572,6 @@
           <t>27</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 10C, 10D, 10E, 11, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -674,11 +579,6 @@
           <t>28</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -686,11 +586,6 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>1, 2, 3A, 3B, 4A, 4B, 5, 6, 7</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -698,11 +593,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -710,11 +600,6 @@
           <t>30</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12, 2, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B, 9C, 9D, 9E</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -722,11 +607,6 @@
           <t>31</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>1, 2A, 2B</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -734,11 +614,6 @@
           <t>32</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6A, 6B</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -746,11 +621,6 @@
           <t>33</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -758,11 +628,6 @@
           <t>34</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -770,11 +635,6 @@
           <t>35</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 1A, 1B, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -782,11 +642,6 @@
           <t>4</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>1A1, 1A2, 1B1A, 1B1B, 1B2, 2, 3, 4A1, 4A2, 4B, 5, 6, 7, 8</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -794,11 +649,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>1, 10A, 10B, 11, 12A, 12B, 13, 14A, 14B, 14C, 14D, 14E, 15A, 15B, 15C, 16A, 16B, 17, 18, 19, 2, 20, 3, 4, 5, 6A, 6B1, 6B2, 6C, 6D1, 6D2, 7A, 7B, 8, 9</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -806,11 +656,6 @@
           <t>6</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -818,11 +663,6 @@
           <t>7</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -830,21 +670,11 @@
           <t>8</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>1, 10, 11A, 11B, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
           <t>9</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>10, 11, 12, 13, 14, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 32 village workbooks (rw-rtx-3070 2026-10-09T15:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Arikathurai_13.34632_80.126.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Arikathurai_13.34632_80.126.xlsx
@@ -614,6 +614,11 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 14, 15, 16, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -621,6 +626,11 @@
           <t>24</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -628,6 +638,11 @@
           <t>25</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>1, 10, 2, 3, 4, 5A, 5B, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -635,6 +650,11 @@
           <t>26</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -642,6 +662,11 @@
           <t>27</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 10D, 10E, 11, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -649,6 +674,11 @@
           <t>28</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -656,6 +686,11 @@
           <t>29</t>
         </is>
       </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>1, 2, 3A, 3B, 4A, 4B, 5, 6, 7</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -663,6 +698,11 @@
           <t>3</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -670,6 +710,11 @@
           <t>30</t>
         </is>
       </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 2, 3, 4A, 4B, 5, 6, 7, 8, 9A, 9B, 9C, 9D, 9E</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -677,6 +722,11 @@
           <t>31</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -684,11 +734,21 @@
           <t>32</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6A, 6B</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
           <t>33</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
progress: 33 village workbooks (rw-rtx-3070 2026-10-09T21:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Arikathurai_13.34632_80.126.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Arikathurai_13.34632_80.126.xlsx
@@ -758,6 +758,11 @@
           <t>34</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -765,6 +770,11 @@
           <t>35</t>
         </is>
       </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2, 3A, 3B, 3C, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -772,6 +782,11 @@
           <t>4</t>
         </is>
       </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B1A, 1B1B, 1B2, 2, 3, 4A1, 4A2, 4B, 5, 6, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -779,6 +794,11 @@
           <t>5</t>
         </is>
       </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12A, 12B, 13, 14A, 14B, 14C, 14D, 14E, 15A, 15B, 15C, 16A, 16B, 17, 18, 19, 2, 20, 3, 4, 5, 6A, 6B1, 6B2, 6C, 6D1, 6D2, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -786,6 +806,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -793,6 +818,11 @@
           <t>7</t>
         </is>
       </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -800,11 +830,21 @@
           <t>8</t>
         </is>
       </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
           <t>9</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>